<commit_message>
Adjusted 2011 height data analysis
</commit_message>
<xml_diff>
--- a/tables/all_model_results.xlsx
+++ b/tables/all_model_results.xlsx
@@ -561,28 +561,28 @@
         </is>
       </c>
       <c r="C2">
-        <v>1.7305</v>
+        <v>1.73</v>
       </c>
       <c r="D2">
-        <v>0.0974</v>
+        <v>0.0979</v>
       </c>
       <c r="E2">
-        <v>1.5375</v>
+        <v>1.5394</v>
       </c>
       <c r="F2">
-        <v>1.9195</v>
+        <v>1.9205</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
       </c>
       <c r="H2">
-        <v>464.32</v>
+        <v>464.08</v>
       </c>
       <c r="I2">
-        <v>365.29</v>
+        <v>366.2</v>
       </c>
       <c r="J2">
-        <v>581.76</v>
+        <v>582.47</v>
       </c>
     </row>
     <row r="3">
@@ -597,16 +597,16 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.423</v>
+        <v>0.4231</v>
       </c>
       <c r="D3">
-        <v>0.0247</v>
+        <v>0.0249</v>
       </c>
       <c r="E3">
-        <v>0.3748</v>
+        <v>0.3743</v>
       </c>
       <c r="F3">
-        <v>0.4721</v>
+        <v>0.472</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
@@ -615,10 +615,10 @@
         <v>52.66</v>
       </c>
       <c r="I3">
-        <v>45.47</v>
+        <v>45.4</v>
       </c>
       <c r="J3">
-        <v>60.34</v>
+        <v>60.32</v>
       </c>
     </row>
     <row r="4">
@@ -633,28 +633,28 @@
         </is>
       </c>
       <c r="C4">
-        <v>-0.0509</v>
+        <v>-0.0508</v>
       </c>
       <c r="D4">
-        <v>0.0201</v>
+        <v>0.0197</v>
       </c>
       <c r="E4">
-        <v>-0.09039999999999999</v>
+        <v>-0.0895</v>
       </c>
       <c r="F4">
-        <v>-0.0113</v>
+        <v>-0.0123</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
       </c>
       <c r="H4">
-        <v>-4.97</v>
+        <v>-4.95</v>
       </c>
       <c r="I4">
-        <v>-8.640000000000001</v>
+        <v>-8.56</v>
       </c>
       <c r="J4">
-        <v>-1.13</v>
+        <v>-1.23</v>
       </c>
     </row>
     <row r="5">
@@ -669,28 +669,28 @@
         </is>
       </c>
       <c r="C5">
-        <v>-0.1167</v>
+        <v>-0.1168</v>
       </c>
       <c r="D5">
-        <v>0.0216</v>
+        <v>0.0213</v>
       </c>
       <c r="E5">
         <v>-0.1595</v>
       </c>
       <c r="F5">
-        <v>-0.0751</v>
+        <v>-0.07539999999999999</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
       </c>
       <c r="H5">
-        <v>-11.02</v>
+        <v>-11.03</v>
       </c>
       <c r="I5">
         <v>-14.74</v>
       </c>
       <c r="J5">
-        <v>-7.23</v>
+        <v>-7.26</v>
       </c>
     </row>
     <row r="6">
@@ -705,28 +705,28 @@
         </is>
       </c>
       <c r="C6">
-        <v>1.3134</v>
+        <v>1.3127</v>
       </c>
       <c r="D6">
-        <v>0.189</v>
+        <v>0.1843</v>
       </c>
       <c r="E6">
-        <v>0.9394</v>
+        <v>0.9554</v>
       </c>
       <c r="F6">
-        <v>1.6885</v>
+        <v>1.6811</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
       </c>
       <c r="H6">
-        <v>271.88</v>
+        <v>271.62</v>
       </c>
       <c r="I6">
-        <v>155.85</v>
+        <v>159.97</v>
       </c>
       <c r="J6">
-        <v>441.12</v>
+        <v>437.14</v>
       </c>
     </row>
     <row r="7">
@@ -741,28 +741,28 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.3637</v>
+        <v>0.3636</v>
       </c>
       <c r="D7">
-        <v>0.0481</v>
+        <v>0.0468</v>
       </c>
       <c r="E7">
-        <v>0.2687</v>
+        <v>0.2698</v>
       </c>
       <c r="F7">
-        <v>0.4585</v>
+        <v>0.454</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
       </c>
       <c r="H7">
-        <v>43.86</v>
+        <v>43.85</v>
       </c>
       <c r="I7">
-        <v>30.83</v>
+        <v>30.97</v>
       </c>
       <c r="J7">
-        <v>58.18</v>
+        <v>57.45</v>
       </c>
     </row>
     <row r="8">
@@ -777,28 +777,28 @@
         </is>
       </c>
       <c r="C8">
-        <v>-0.0008</v>
+        <v>0.0001</v>
       </c>
       <c r="D8">
-        <v>0.0453</v>
+        <v>0.046</v>
       </c>
       <c r="E8">
-        <v>-0.089</v>
+        <v>-0.0897</v>
       </c>
       <c r="F8">
-        <v>0.08840000000000001</v>
+        <v>0.0898</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>-0.08</v>
+        <v>0.01</v>
       </c>
       <c r="I8">
-        <v>-8.52</v>
+        <v>-8.58</v>
       </c>
       <c r="J8">
-        <v>9.25</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="9">
@@ -813,28 +813,28 @@
         </is>
       </c>
       <c r="C9">
-        <v>-0.0566</v>
+        <v>-0.0556</v>
       </c>
       <c r="D9">
-        <v>0.0464</v>
+        <v>0.046</v>
       </c>
       <c r="E9">
-        <v>-0.1477</v>
+        <v>-0.146</v>
       </c>
       <c r="F9">
-        <v>0.0354</v>
+        <v>0.0337</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
       </c>
       <c r="H9">
-        <v>-5.5</v>
+        <v>-5.41</v>
       </c>
       <c r="I9">
-        <v>-13.73</v>
+        <v>-13.58</v>
       </c>
       <c r="J9">
-        <v>3.6</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="10">
@@ -849,28 +849,28 @@
         </is>
       </c>
       <c r="C10">
-        <v>-1.2881</v>
+        <v>-1.2864</v>
       </c>
       <c r="D10">
-        <v>0.351</v>
+        <v>0.3531</v>
       </c>
       <c r="E10">
-        <v>-1.996</v>
+        <v>-1.9976</v>
       </c>
       <c r="F10">
-        <v>-0.6032999999999999</v>
+        <v>-0.6067</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
       </c>
       <c r="H10">
-        <v>-72.42</v>
+        <v>-72.37</v>
       </c>
       <c r="I10">
-        <v>-86.41</v>
+        <v>-86.43000000000001</v>
       </c>
       <c r="J10">
-        <v>-45.3</v>
+        <v>-45.49</v>
       </c>
     </row>
     <row r="11">
@@ -885,28 +885,28 @@
         </is>
       </c>
       <c r="C11">
-        <v>1.531</v>
+        <v>1.5309</v>
       </c>
       <c r="D11">
-        <v>0.0895</v>
+        <v>0.0898</v>
       </c>
       <c r="E11">
-        <v>1.3581</v>
+        <v>1.3569</v>
       </c>
       <c r="F11">
-        <v>1.7106</v>
+        <v>1.7117</v>
       </c>
       <c r="G11" t="b">
         <v>1</v>
       </c>
       <c r="H11">
-        <v>362.3</v>
+        <v>362.25</v>
       </c>
       <c r="I11">
-        <v>288.87</v>
+        <v>288.43</v>
       </c>
       <c r="J11">
-        <v>453.21</v>
+        <v>453.84</v>
       </c>
     </row>
     <row r="12">
@@ -921,28 +921,28 @@
         </is>
       </c>
       <c r="C12">
-        <v>-0.1053</v>
+        <v>-0.106</v>
       </c>
       <c r="D12">
-        <v>0.0716</v>
+        <v>0.07149999999999999</v>
       </c>
       <c r="E12">
-        <v>-0.2468</v>
+        <v>-0.2495</v>
       </c>
       <c r="F12">
-        <v>0.0351</v>
+        <v>0.0345</v>
       </c>
       <c r="G12" t="b">
         <v>0</v>
       </c>
       <c r="H12">
-        <v>-9.99</v>
+        <v>-10.06</v>
       </c>
       <c r="I12">
-        <v>-21.87</v>
+        <v>-22.08</v>
       </c>
       <c r="J12">
-        <v>3.57</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="13">
@@ -957,16 +957,16 @@
         </is>
       </c>
       <c r="C13">
-        <v>-0.2528</v>
+        <v>-0.2529</v>
       </c>
       <c r="D13">
-        <v>0.0771</v>
+        <v>0.077</v>
       </c>
       <c r="E13">
-        <v>-0.4068</v>
+        <v>-0.4058</v>
       </c>
       <c r="F13">
-        <v>-0.1058</v>
+        <v>-0.1057</v>
       </c>
       <c r="G13" t="b">
         <v>1</v>
@@ -975,10 +975,10 @@
         <v>-22.34</v>
       </c>
       <c r="I13">
-        <v>-33.42</v>
+        <v>-33.35</v>
       </c>
       <c r="J13">
-        <v>-10.04</v>
+        <v>-10.03</v>
       </c>
     </row>
     <row r="14">
@@ -993,28 +993,28 @@
         </is>
       </c>
       <c r="C14">
-        <v>-0.7345</v>
+        <v>-0.7448</v>
       </c>
       <c r="D14">
-        <v>0.5034</v>
+        <v>0.5012</v>
       </c>
       <c r="E14">
-        <v>-1.7267</v>
+        <v>-1.7458</v>
       </c>
       <c r="F14">
-        <v>0.2405</v>
+        <v>0.2211</v>
       </c>
       <c r="G14" t="b">
         <v>0</v>
       </c>
       <c r="H14">
-        <v>-52.03</v>
+        <v>-52.52</v>
       </c>
       <c r="I14">
-        <v>-82.20999999999999</v>
+        <v>-82.55</v>
       </c>
       <c r="J14">
-        <v>27.19</v>
+        <v>24.75</v>
       </c>
     </row>
     <row r="15">
@@ -1029,28 +1029,28 @@
         </is>
       </c>
       <c r="C15">
-        <v>1.7609</v>
+        <v>1.7642</v>
       </c>
       <c r="D15">
-        <v>0.1284</v>
+        <v>0.1277</v>
       </c>
       <c r="E15">
-        <v>1.5144</v>
+        <v>1.5181</v>
       </c>
       <c r="F15">
-        <v>2.0124</v>
+        <v>2.0201</v>
       </c>
       <c r="G15" t="b">
         <v>1</v>
       </c>
       <c r="H15">
-        <v>481.79</v>
+        <v>483.68</v>
       </c>
       <c r="I15">
-        <v>354.68</v>
+        <v>356.35</v>
       </c>
       <c r="J15">
-        <v>648.13</v>
+        <v>653.92</v>
       </c>
     </row>
     <row r="16">
@@ -1065,28 +1065,28 @@
         </is>
       </c>
       <c r="C16">
-        <v>-0.07580000000000001</v>
+        <v>-0.07729999999999999</v>
       </c>
       <c r="D16">
-        <v>0.1007</v>
+        <v>0.1016</v>
       </c>
       <c r="E16">
-        <v>-0.273</v>
+        <v>-0.2796</v>
       </c>
       <c r="F16">
-        <v>0.1198</v>
+        <v>0.12</v>
       </c>
       <c r="G16" t="b">
         <v>0</v>
       </c>
       <c r="H16">
-        <v>-7.3</v>
+        <v>-7.44</v>
       </c>
       <c r="I16">
-        <v>-23.89</v>
+        <v>-24.39</v>
       </c>
       <c r="J16">
-        <v>12.72</v>
+        <v>12.75</v>
       </c>
     </row>
     <row r="17">
@@ -1101,28 +1101,28 @@
         </is>
       </c>
       <c r="C17">
-        <v>-0.2993</v>
+        <v>-0.2998</v>
       </c>
       <c r="D17">
-        <v>0.1069</v>
+        <v>0.1073</v>
       </c>
       <c r="E17">
-        <v>-0.5145</v>
+        <v>-0.5143</v>
       </c>
       <c r="F17">
-        <v>-0.0949</v>
+        <v>-0.094</v>
       </c>
       <c r="G17" t="b">
         <v>1</v>
       </c>
       <c r="H17">
-        <v>-25.87</v>
+        <v>-25.91</v>
       </c>
       <c r="I17">
-        <v>-40.22</v>
+        <v>-40.21</v>
       </c>
       <c r="J17">
-        <v>-9.06</v>
+        <v>-8.970000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -1137,28 +1137,28 @@
         </is>
       </c>
       <c r="C18">
-        <v>-0.4866</v>
+        <v>-0.4874</v>
       </c>
       <c r="D18">
-        <v>0.041</v>
+        <v>0.0414</v>
       </c>
       <c r="E18">
-        <v>-0.5674</v>
+        <v>-0.5699</v>
       </c>
       <c r="F18">
-        <v>-0.4069</v>
+        <v>-0.4077</v>
       </c>
       <c r="G18" t="b">
         <v>1</v>
       </c>
       <c r="H18">
-        <v>-38.53</v>
+        <v>-38.58</v>
       </c>
       <c r="I18">
-        <v>-43.3</v>
+        <v>-43.44</v>
       </c>
       <c r="J18">
-        <v>-33.43</v>
+        <v>-33.48</v>
       </c>
     </row>
     <row r="19">
@@ -1173,28 +1173,28 @@
         </is>
       </c>
       <c r="C19">
-        <v>-0.0348</v>
+        <v>-0.0346</v>
       </c>
       <c r="D19">
-        <v>0.0374</v>
+        <v>0.0376</v>
       </c>
       <c r="E19">
-        <v>-0.1084</v>
+        <v>-0.1094</v>
       </c>
       <c r="F19">
-        <v>0.0374</v>
+        <v>0.039</v>
       </c>
       <c r="G19" t="b">
         <v>0</v>
       </c>
       <c r="H19">
-        <v>-3.42</v>
+        <v>-3.4</v>
       </c>
       <c r="I19">
-        <v>-10.27</v>
+        <v>-10.37</v>
       </c>
       <c r="J19">
-        <v>3.81</v>
+        <v>3.98</v>
       </c>
     </row>
     <row r="20">
@@ -1209,28 +1209,28 @@
         </is>
       </c>
       <c r="C20">
-        <v>-0.07290000000000001</v>
+        <v>-0.0728</v>
       </c>
       <c r="D20">
-        <v>0.0385</v>
+        <v>0.0387</v>
       </c>
       <c r="E20">
-        <v>-0.148</v>
+        <v>-0.1487</v>
       </c>
       <c r="F20">
-        <v>0.002</v>
+        <v>0.0035</v>
       </c>
       <c r="G20" t="b">
         <v>0</v>
       </c>
       <c r="H20">
-        <v>-7.03</v>
+        <v>-7.02</v>
       </c>
       <c r="I20">
-        <v>-13.75</v>
+        <v>-13.82</v>
       </c>
       <c r="J20">
-        <v>0.2</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="21">
@@ -1245,28 +1245,28 @@
         </is>
       </c>
       <c r="C21">
-        <v>-0.8023</v>
+        <v>-0.8028</v>
       </c>
       <c r="D21">
-        <v>0.054</v>
+        <v>0.0531</v>
       </c>
       <c r="E21">
-        <v>-0.9104</v>
+        <v>-0.9081</v>
       </c>
       <c r="F21">
-        <v>-0.6987</v>
+        <v>-0.6997</v>
       </c>
       <c r="G21" t="b">
         <v>1</v>
       </c>
       <c r="H21">
-        <v>-55.17</v>
+        <v>-55.19</v>
       </c>
       <c r="I21">
-        <v>-59.76</v>
+        <v>-59.67</v>
       </c>
       <c r="J21">
-        <v>-50.28</v>
+        <v>-50.33</v>
       </c>
     </row>
     <row r="22">
@@ -1281,28 +1281,28 @@
         </is>
       </c>
       <c r="C22">
-        <v>-0.0417</v>
+        <v>-0.0405</v>
       </c>
       <c r="D22">
-        <v>0.0572</v>
+        <v>0.0553</v>
       </c>
       <c r="E22">
-        <v>-0.1538</v>
+        <v>-0.1495</v>
       </c>
       <c r="F22">
-        <v>0.0697</v>
+        <v>0.0669</v>
       </c>
       <c r="G22" t="b">
         <v>0</v>
       </c>
       <c r="H22">
-        <v>-4.09</v>
+        <v>-3.97</v>
       </c>
       <c r="I22">
-        <v>-14.26</v>
+        <v>-13.89</v>
       </c>
       <c r="J22">
-        <v>7.21</v>
+        <v>6.92</v>
       </c>
     </row>
     <row r="23">
@@ -1317,28 +1317,28 @@
         </is>
       </c>
       <c r="C23">
-        <v>-0.07480000000000001</v>
+        <v>-0.0733</v>
       </c>
       <c r="D23">
-        <v>0.0613</v>
+        <v>0.0594</v>
       </c>
       <c r="E23">
-        <v>-0.1966</v>
+        <v>-0.1908</v>
       </c>
       <c r="F23">
-        <v>0.0431</v>
+        <v>0.0422</v>
       </c>
       <c r="G23" t="b">
         <v>0</v>
       </c>
       <c r="H23">
-        <v>-7.2</v>
+        <v>-7.07</v>
       </c>
       <c r="I23">
-        <v>-17.85</v>
+        <v>-17.37</v>
       </c>
       <c r="J23">
-        <v>4.41</v>
+        <v>4.31</v>
       </c>
     </row>
   </sheetData>
@@ -2259,28 +2259,28 @@
         </is>
       </c>
       <c r="C2">
-        <v>1.746</v>
+        <v>1.7874</v>
       </c>
       <c r="D2">
-        <v>0.0597</v>
+        <v>0.0587</v>
       </c>
       <c r="E2">
-        <v>1.6292</v>
+        <v>1.6732</v>
       </c>
       <c r="F2">
-        <v>1.8619</v>
+        <v>1.9023</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
       </c>
       <c r="H2">
-        <v>473.17</v>
+        <v>497.4</v>
       </c>
       <c r="I2">
-        <v>409.98</v>
+        <v>432.94</v>
       </c>
       <c r="J2">
-        <v>543.59</v>
+        <v>570.12</v>
       </c>
     </row>
     <row r="3">
@@ -2298,10 +2298,10 @@
         <v>0.3996</v>
       </c>
       <c r="D3">
-        <v>0.0148</v>
+        <v>0.0147</v>
       </c>
       <c r="E3">
-        <v>0.3706</v>
+        <v>0.3705</v>
       </c>
       <c r="F3">
         <v>0.4286</v>
@@ -2310,10 +2310,10 @@
         <v>1</v>
       </c>
       <c r="H3">
-        <v>49.12</v>
+        <v>49.13</v>
       </c>
       <c r="I3">
-        <v>44.86</v>
+        <v>44.85</v>
       </c>
       <c r="J3">
         <v>53.51</v>
@@ -2327,32 +2327,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>h2_2011_categoryremaineduninfested</t>
+          <t>h2_2011_categorygainedinfestation</t>
         </is>
       </c>
       <c r="C4">
-        <v>0.0416</v>
+        <v>-0.0418</v>
       </c>
       <c r="D4">
         <v>0.0146</v>
       </c>
       <c r="E4">
-        <v>0.0128</v>
+        <v>-0.0703</v>
       </c>
       <c r="F4">
-        <v>0.0697</v>
+        <v>-0.0126</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
       </c>
       <c r="H4">
-        <v>4.25</v>
+        <v>-4.09</v>
       </c>
       <c r="I4">
-        <v>1.29</v>
+        <v>-6.79</v>
       </c>
       <c r="J4">
-        <v>7.21</v>
+        <v>-1.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New MM transformation for 2011 height model
</commit_message>
<xml_diff>
--- a/tables/all_model_results.xlsx
+++ b/tables/all_model_results.xlsx
@@ -2995,7 +2995,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -3048,20 +3048,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Intercept</t>
+          <t>Vm_Intercept</t>
         </is>
       </c>
       <c r="C2">
-        <v>1.79</v>
+        <v>3.96</v>
       </c>
       <c r="D2">
-        <v>0.0587</v>
+        <v>0.109</v>
       </c>
       <c r="E2">
-        <v>1.67</v>
+        <v>3.83</v>
       </c>
       <c r="F2">
-        <v>1.9</v>
+        <v>4.15</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -3069,7 +3069,7 @@
         </is>
       </c>
       <c r="H2">
-        <v>497</v>
+        <v>5170</v>
       </c>
     </row>
     <row r="3">
@@ -3080,28 +3080,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>log_dbh_2011</t>
+          <t>Vm_h2_2011_categorygainedinfestation</t>
         </is>
       </c>
       <c r="C3">
-        <v>0.4</v>
+        <v>-0.133</v>
       </c>
       <c r="D3">
-        <v>0.0147</v>
+        <v>0.162</v>
       </c>
       <c r="E3">
-        <v>0.371</v>
+        <v>-0.304</v>
       </c>
       <c r="F3">
-        <v>0.429</v>
+        <v>0.0723</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H3">
-        <v>49.1</v>
+        <v>-12.4</v>
       </c>
     </row>
     <row r="4">
@@ -3112,20 +3112,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>h2_2011_categorygainedinfestation</t>
+          <t>x_Intercept</t>
         </is>
       </c>
       <c r="C4">
-        <v>-0.0418</v>
+        <v>0.907</v>
       </c>
       <c r="D4">
-        <v>0.0146</v>
+        <v>0.09130000000000001</v>
       </c>
       <c r="E4">
-        <v>-0.0703</v>
+        <v>0.73</v>
       </c>
       <c r="F4">
-        <v>-0.0126</v>
+        <v>1.07</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -3133,7 +3133,103 @@
         </is>
       </c>
       <c r="H4">
-        <v>-4.09</v>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>H2 height 2011 — log(height 2011)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>x_h2_2011_categorygainedinfestation</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>0.298</v>
+      </c>
+      <c r="D5">
+        <v>0.106</v>
+      </c>
+      <c r="E5">
+        <v>0.0544</v>
+      </c>
+      <c r="F5">
+        <v>0.489</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5">
+        <v>34.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>H2 height 2011 — log(height 2011)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>K_Intercept</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>27.6</v>
+      </c>
+      <c r="D6">
+        <v>4.96</v>
+      </c>
+      <c r="E6">
+        <v>19.7</v>
+      </c>
+      <c r="F6">
+        <v>39</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H6">
+        <v>98400000000000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>H2 height 2011 — log(height 2011)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>K_h2_2011_categorygainedinfestation</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>38.9</v>
+      </c>
+      <c r="D7">
+        <v>15.3</v>
+      </c>
+      <c r="E7">
+        <v>12.4</v>
+      </c>
+      <c r="F7">
+        <v>71.8</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7">
+        <v>7.6E+18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>